<commit_message>
updated for KPI doctypes
</commit_message>
<xml_diff>
--- a/auto_repair/public/www/assets/xlsx/poas.xlsx
+++ b/auto_repair/public/www/assets/xlsx/poas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abees\Documents\sic\auto-repair-erp\web\src\assets\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4882E389-B247-40F8-91AE-F9022C3BAE9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35BDC3A-9439-4329-9340-ED476F21C816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{8CDF2226-9A4B-4898-83BA-55E8F32B23C5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{8CDF2226-9A4B-4898-83BA-55E8F32B23C5}"/>
   </bookViews>
   <sheets>
     <sheet name="Phases" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="8">
   <si>
     <t>subject</t>
   </si>
@@ -61,6 +61,9 @@
   </si>
   <si>
     <t>parent_tracking_id</t>
+  </si>
+  <si>
+    <t>remarks</t>
   </si>
 </sst>
 </file>
@@ -68,7 +71,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd;@"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -104,7 +107,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -480,20 +483,21 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2EB4C9A7-595A-454D-AD5E-6DCC61FFEB06}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" style="1" customWidth="1"/>
     <col min="2" max="2" width="15.88671875" style="1" customWidth="1"/>
     <col min="3" max="3" width="16" style="1" customWidth="1"/>
     <col min="4" max="4" width="32.21875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="14.5546875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="15.5546875" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="1"/>
+    <col min="5" max="5" width="15.5546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="15.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14.5546875" style="2" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -507,12 +511,15 @@
         <v>1</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="H1" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>